<commit_message>
fix: complete bilingual localization audit
</commit_message>
<xml_diff>
--- a/prototype_baseline/review/materialized_dataset_review.xlsx
+++ b/prototype_baseline/review/materialized_dataset_review.xlsx
@@ -1748,7 +1748,7 @@
         <x:v>involved</x:v>
       </x:c>
       <x:c r="I7" s="4" t="str">
-        <x:v>The patient is unconscious and cannot provide an anamnesis. Only accessible prior records and current physical-examination or encounter findings may be used.</x:v>
+        <x:v>The patient is unconscious and cannot provide a medical history. Only accessible prior records and current physical-examination or encounter findings may be used.</x:v>
       </x:c>
       <x:c r="J7" s="6" t="b">
         <x:v>1</x:v>
@@ -2088,7 +2088,7 @@
         <x:v>record</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
-        <x:v>Generalized anxiety disorder is documented.</x:v>
+        <x:v>Generalised anxiety disorder is documented.</x:v>
       </x:c>
       <x:c r="G14" s="4" t="n">
         <x:v>3</x:v>
@@ -2249,7 +2249,7 @@
         <x:v>physical_exam</x:v>
       </x:c>
       <x:c r="F21" s="4" t="str">
-        <x:v>Localized low-back pain without leg radiation is recorded; no underlying diagnosis has been established for this finding.</x:v>
+        <x:v>Localised low-back pain without leg radiation is recorded; no underlying diagnosis has been established for this finding.</x:v>
       </x:c>
       <x:c r="G21" s="4" t="n">
         <x:v>5</x:v>
@@ -2387,7 +2387,7 @@
         <x:v>physical_exam</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
-        <x:v>The patient is unconscious and cannot provide an anamnesis at the represented encounter.</x:v>
+        <x:v>The patient is unconscious and cannot provide a medical history at the represented encounter.</x:v>
       </x:c>
       <x:c r="G27" s="4" t="n">
         <x:v>1</x:v>
@@ -2456,7 +2456,7 @@
         <x:v>record</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
-        <x:v>Generalized idiopathic epilepsy is documented; the record does not establish it as the cause of the current unconsciousness.</x:v>
+        <x:v>Generalised idiopathic epilepsy is documented; the record does not establish it as the cause of the current unconsciousness.</x:v>
       </x:c>
       <x:c r="G30" s="4" t="n">
         <x:v>4</x:v>
@@ -2841,7 +2841,7 @@
         <x:v>Anxiety coding task</x:v>
       </x:c>
       <x:c r="F10" s="4" t="str">
-        <x:v>The record explicitly states generalized anxiety disorder. Select the best supported code.</x:v>
+        <x:v>The record explicitly states generalised anxiety disorder. Select the best supported code.</x:v>
       </x:c>
       <x:c r="G10" s="4" t="str">
         <x:v>learner_visible</x:v>
@@ -2991,7 +2991,7 @@
         <x:v>Current-finding coding task</x:v>
       </x:c>
       <x:c r="F15" s="4" t="str">
-        <x:v>During assessment the patient reports localized low-back pain without leg radiation; no underlying diagnosis is established. Which of the displayed choices best represents the documented finding?</x:v>
+        <x:v>During assessment the patient reports localised low-back pain without leg radiation; no underlying diagnosis is established. Which of the displayed choices best represents the documented finding?</x:v>
       </x:c>
       <x:c r="G15" s="4" t="str">
         <x:v>learner_visible</x:v>
@@ -3231,7 +3231,7 @@
         <x:v>Prior epilepsy-record coding task</x:v>
       </x:c>
       <x:c r="F23" s="4" t="str">
-        <x:v>The accessible prior record explicitly states generalized idiopathic epilepsy. No status epilepticus is represented. Select the best supported code for that chronic diagnosis.</x:v>
+        <x:v>The accessible prior record explicitly states generalised idiopathic epilepsy. No status epilepticus is represented. Select the best supported code for that chronic diagnosis.</x:v>
       </x:c>
       <x:c r="G23" s="4" t="str">
         <x:v>learner_visible</x:v>

</xml_diff>